<commit_message>
Atualização do módulo microrregião.
</commit_message>
<xml_diff>
--- a/dados/tradutor_gempack.xlsx
+++ b/dados/tradutor_gempack.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\desenvolvimentos\apps\gd_impacta_mg\dados\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E6A052F-7F79-4136-A779-F2749ACE7D0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A21BC476-8FA7-4FAB-99E2-372FA3AA739C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" activeTab="3" xr2:uid="{98DCC10F-1E1E-46D0-8590-C8CA17A0E6A3}"/>
+    <workbookView xWindow="19515" yWindow="4650" windowWidth="21780" windowHeight="20985" activeTab="3" xr2:uid="{98DCC10F-1E1E-46D0-8590-C8CA17A0E6A3}"/>
   </bookViews>
   <sheets>
     <sheet name="scn" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="318">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="482" uniqueCount="319">
   <si>
     <t>Agricultura, inclusive o apoio à agricultura e a pós-colheita</t>
   </si>
@@ -993,6 +993,9 @@
   </si>
   <si>
     <t>resultado</t>
+  </si>
+  <si>
+    <t>São João del Rei</t>
   </si>
 </sst>
 </file>
@@ -3544,7 +3547,7 @@
         <v>305</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>103</v>
+        <v>318</v>
       </c>
     </row>
     <row r="57" spans="1:2" x14ac:dyDescent="0.25">

</xml_diff>